<commit_message>
Prepare registry-stack v0.8.4 beta-10
Signed-off-by: Jeremi Joslin <jeremi@joslin.fr>
</commit_message>
<xml_diff>
--- a/lab/data/social-protection/social-protection.xlsx
+++ b/lab/data/social-protection/social-protection.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-06-17T12:59:47Z</t>
+          <t>2026-07-02T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-06-17T12:59:47Z</t>
+          <t>2026-07-02T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-06-19T12:59:47Z</t>
+          <t>2026-07-04T09:45:02Z</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-06-17T12:59:47Z</t>
+          <t>2026-07-02T09:45:02Z</t>
         </is>
       </c>
     </row>

</xml_diff>